<commit_message>
fix(output): add blank separator row between scalar and table sections in xlsx
User-corrected fixture 04 control file revealed that a blank row should
separate the scalar var: section from the table: section when both are present.
Added the separator in xlsx_writer, updated the test, and regenerated all
mixed-content fixture control files (03-22) to match.

All 4 user-curated control files (01-04) now match exactly. 1484 tests pass.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/03_purchase_order/data-export-control.xlsx
+++ b/tests/fixtures/03_purchase_order/data-export-control.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -593,143 +593,144 @@
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>table:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>HEADER</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>row.item</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>row.desc</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>row.qty</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>row.price</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>row.total</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="6" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>DATA</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Laptop</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Dell XPS 15</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="G7" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H7" s="5" t="n">
         <v>2400</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="8" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>DATA</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Monitor Stand</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F8" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G8" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H8" s="7" t="n">
         <v>180</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>DATA</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Dock</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>USB-C Hub</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F9" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G9" s="5" t="n">
         <v>75</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H9" s="5" t="n">
         <v>450</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="10" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="n"/>
+      <c r="B10" s="9" t="n"/>
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>FOOTER</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="9" t="n">
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n">
         <v>3030</v>
       </c>
     </row>

</xml_diff>